<commit_message>
sync 2 wandb runs from TRM_CR
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -494,8 +494,52 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp002_result.png")</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exp11_nsup4_8_16_mix_10000_000959_stage1_0qr1zveh</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="F3">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp11_nsup4_8_16_mix_10000_000959_stage1_0qr1zveh.png")</f>
+        <v/>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/0qr1zveh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>exp12_nsup16_curriculum_10000_resume_001054_stage1_h1o6ig1c</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp12_nsup16_curriculum_10000_resume_001054_stage1_h1o6ig1c.png")</f>
+        <v/>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/h1o6ig1c</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add 2 run(s) to index: cr_0413_baseline_220918_stage2, cp_0413_cr_trace_mix_164606_stage2
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -527,9 +527,6 @@
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp12_nsup16_curriculum_10000_resume_001054_stage1_h1o6ig1c.png")</f>
         <v/>
@@ -539,7 +536,64 @@
           <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/h1o6ig1c</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cr_0413_baseline_220918_stage2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>768</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cr_0413_baseline_220918</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="100" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cp_0413_cr_trace_mix_164606_stage2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>768</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cp_0413_cr_trace_mix_164606_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cp_0413_cr_trace_mix_164606</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
cleanup: keep only the 2 real W&B runs in main index
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -26,12 +26,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -422,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -473,127 +468,68 @@
     <row r="2" ht="100" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>exp002</t>
+          <t>cr_0413_baseline_220918_stage2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="D2" t="n">
-        <v>128</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.88</v>
-      </c>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>768</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp002_result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cr_0413_baseline_220918</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>exp11_nsup4_8_16_mix_10000_000959_stage1_0qr1zveh</t>
+          <t>cp_0413_cr_trace_mix_164606_stage2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>768</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp11_nsup4_8_16_mix_10000_000959_stage1_0qr1zveh.png")</f>
-        <v/>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/0qr1zveh</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>exp12_nsup16_curriculum_10000_resume_001054_stage1_h1o6ig1c</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="F4">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/main/exp12_nsup16_curriculum_10000_resume_001054_stage1_h1o6ig1c.png")</f>
-        <v/>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/h1o6ig1c</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>cr_0413_baseline_220918_stage2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D5" t="n">
-        <v>768</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cr_0413_baseline_220918</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="100" customHeight="1">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>cp_0413_cr_trace_mix_164606_stage2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D6" t="n">
-        <v>768</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cp_0413_cr_trace_mix_164606_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cp_0413_cr_trace_mix_164606</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
remove cp_0413 from index (branch deleted)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -498,39 +498,6 @@
       </c>
       <c r="H2" t="inlineStr"/>
     </row>
-    <row r="3" ht="100" customHeight="1">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>cp_0413_cr_trace_mix_164606_stage2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0.0001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>768</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cp_0413_cr_trace_mix_164606_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cp_0413_cr_trace_mix_164606</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
new schema: Date, H_cycles, L_cycles, max_halt_steps, photo, wandb_id
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,86 +417,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>H_cycles</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>lr</t>
+          <t>L_cycles</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>bs</t>
+          <t>max_halt_steps</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>best_acc</t>
+          <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>PhotoURL</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>W&amp;B</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>wandb_id</t>
         </is>
       </c>
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cr_0413_baseline_220918_stage2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0.0001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>768</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2">
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://wandb.ai/sfu-tai-lab-zhe/TRM_CR/runs/cr_0413_baseline_220918</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>cr_0413_baseline_220918</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
schema: drop Date, add nsup32/nsup64 photo columns
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,64 +417,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>H_cycles</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>H_cycles</t>
+          <t>L_cycles</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>L_cycles</t>
+          <t>max_halt_steps</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>max_halt_steps</t>
+          <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>exact_acc @ halt_or_nsup 16</t>
+          <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>exact_acc @ halt_or_nsup 64</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>wandb_id</t>
         </is>
       </c>
     </row>
     <row r="2" ht="100" customHeight="1">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
         <v>16</v>
       </c>
-      <c r="E2">
+      <c r="D2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>cr_0413_baseline_220918</t>
         </is>

</xml_diff>

<commit_message>
rebuild index with all 6 nsup64 runs; wandb_id moved to first column
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,77 +417,217 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>wandb_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>H_cycles</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>L_cycles</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>max_halt_steps</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>wandb_id</t>
         </is>
       </c>
     </row>
     <row r="2" ht="100" customHeight="1">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cr_0413_baseline_220918</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>16</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>cr_0413_baseline_220918</t>
-        </is>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exp_0413_cr_trace_mix_gaussian_210715</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>exp_0414_bt_004417</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>exp_0414_bt_descendents_015622</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="100" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>exp_0419_cr_baseline_004937</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="100" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>exp_0420_cr_trace_mix_gaussian_dense_141633</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 1 run(s) to index: exp_0421_cr_trace_mix_gaussian_192914
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="5" max="5"/>
@@ -630,6 +630,34 @@
         <v/>
       </c>
     </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>exp_0421_cr_trace_mix_gaussian_192914</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add config_url column to experiments.csv
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -417,12 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,6 +462,11 @@
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>config_url</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -489,6 +495,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -517,6 +528,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="100" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -545,6 +561,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -573,6 +594,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -601,6 +627,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="100" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -629,6 +660,11 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/config/config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="100" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -656,6 +692,11 @@
       <c r="G8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/config/config.yaml</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inline config content (replacing config_url)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -49,9 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,48 +426,48 @@
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>wandb_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>H_cycles</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>L_cycles</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>max_halt_steps</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>config_url</t>
+          <t>config</t>
         </is>
       </c>
     </row>
@@ -474,30 +477,63 @@
           <t>cr_0413_baseline_220918</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
-        <v>16</v>
-      </c>
-      <c r="E2">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F2">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G2">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/config/config.yaml</t>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Baseline, no CR on depth, no CR on data
+#
+# Usage: bash pretrain_cr.sh cr_0413_baseline.yaml
+name: cr_0413_baseline
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 30000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>
@@ -507,30 +543,85 @@
           <t>exp_0413_cr_trace_mix_gaussian_210715</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>16</v>
-      </c>
-      <c r="E3">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F3">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G3">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/config/config.yaml</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Curriculum learning config (gaussian variant).
+#
+# Same hard-gold-path mix as cp_0413_cr_trace_mix, but the intermediate
+# board's empty-cell count is drawn per-sample from a Gaussian instead of
+# being a fixed constant. This smooths the per-stage empty-cell distribution
+# so the transition into the natural stage-3 distribution (~54-58 empties)
+# is less abrupt.
+#
+# Build the curriculum datasets once before training:
+#
+#   python -m dataset.build_curriculum_dataset \
+#     --source-dir data/sudoku-extreme-1k-aug-1000 \
+#     --output-dir data/sudoku-extreme-1k-aug-1000-stage1-hard-gp-gaussian \
+#     --empty-cells-mean 20 --empty-cells-std 5 --hard-only
+#
+#   python -m dataset.build_curriculum_dataset \
+#     --source-dir data/sudoku-extreme-1k-aug-1000 \
+#     --output-dir data/sudoku-extreme-1k-aug-1000-stage2-hard-gp-gaussian \
+#     --empty-cells-mean 40 --empty-cells-std 5 --hard-only
+#
+# Stage 1. hard -&gt; intermediate @ N(20, 5) empty cells; easy/medium unchanged
+# Stage 2. hard -&gt; intermediate @ N(40, 5) empty cells; easy/medium unchanged
+# Stage 3. original dataset (no replacement)
+#
+# Usage: bash pretrain_cr.sh exp_0413_cr_trace_mix_gaussian.yaml
+name: exp_0413_cr_trace_mix_gaussian
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage1-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage2-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 30000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>
@@ -540,30 +631,72 @@
           <t>exp_0414_bt_004417</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E4">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F4">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G4">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/config/config.yaml</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Curriculum learning config (BT)
+#
+# Stage 1. hard -&gt; wrong son of branch guessing node g1; easy/medium unchanged
+# Stage 2. hard -&gt; wrong son of branch guessing node g2; easy/medium unchanged
+# Stage 3. original dataset (no replacement)
+# g1 = last branching guess on gold path (fewer empty cells, deeper)
+# g2 = second-to-last branching guess on gold path (more empty cells, shallower)
+# empty_cell (g1) &lt; empty_cell (g2)
+# empty_cell (wc_1) = empty_cell (g1) - 1
+# empty_cell (wc_2) = empty_cell (g2) - 1
+#
+# Usage: bash pretrain_cr.sh exp_0414_bt.yaml
+name: exp_0414_bt
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000-bt-stage1-hard
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-bt-stage2-hard
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 30000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>
@@ -573,30 +706,77 @@
           <t>exp_0414_bt_descendents_015622</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="n">
-        <v>16</v>
-      </c>
-      <c r="E5">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F5">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G5">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/config/config.yaml</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Curriculum learning config (BT by wrong-subtree depth, hard-only replacement)
+#
+# Stage 1. hard -&gt; wrong child  of g1 (last branching guess on gold path)
+#                  bt-depth=1   (one wrong step)
+#          easy/medium unchanged
+# Stage 2. hard -&gt; wrong grandchild of g2 (second-last branching guess)
+#                  bt-depth=2   (wrong step + one more walk step)
+#          easy/medium unchanged
+# Stage 3. original dataset (no replacement)
+#
+# g1 = last branching guess (deeper, fewer empty cells)
+# g2 = second-to-last branching guess (shallower, more empty cells)
+# Extra walk steps inside the wrong subtree reuse find_one_propagation and
+# MRV guess-cell selection (see utils/sudoku_with_wrong_child.py ::
+# get_wrong_descendants).
+#
+# Usage: bash pretrain_cr.sh exp_0414_bt_descendents.yaml
+name: exp_0414_bt_descendents
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000-bt-s1-d1-hard
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-bt-s2-d2-hard
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 30000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>
@@ -606,30 +786,63 @@
           <t>exp_0419_cr_baseline_004937</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" t="n">
-        <v>16</v>
-      </c>
-      <c r="E6">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F6">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G6">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/config/config.yaml</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Baseline, no CR on depth, no CR on data
+#
+# Usage: bash pretrain_cr.sh exp_0419_cr_baseline.yaml
+name: exp_0419_cr_baseline
+depth:
+  H_cycles: 2
+  L_cycles: 4
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 30000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>
@@ -639,30 +852,160 @@
           <t>exp_0420_cr_trace_mix_gaussian_dense_141633</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>16</v>
-      </c>
-      <c r="E7">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F7">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G7">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/config/config.yaml</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Curriculum learning config (gaussian, dense variant).
+#
+# 20-stage progression with per-sample empty-cell count drawn from a Gaussian
+# N(mean, 5). Stages match build_data.sh — means ramp from 31 to 70 over 20
+# stages (2500 epochs each) for a dense, near-continuous curriculum. Build
+# the curriculum datasets once before training by running:
+#
+#   bash build_data.sh
+#
+# Usage: bash pretrain_cr.sh exp_0420_cr_trace_mix_gaussian_dense.yaml
+name: exp_0420_cr_trace_mix_gaussian_dense
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-31-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-35-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-39-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-42-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-45-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-47-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-49-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-51-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-53-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-55-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-57-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-58-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-60-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-61-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-63-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-64-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-66-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-67-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-68-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000-hard-gp-gaussian-empty_cell-70-5
+    nsup: 16
+    num_epochs: 2500
+    batch_size: 768
+    eval_interval: 500
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 500
+</t>
         </is>
       </c>
     </row>
@@ -672,30 +1015,107 @@
           <t>exp_0421_cr_trace_mix_gaussian_192914</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F8">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/config/config.yaml</t>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Curriculum learning config (gaussian variant).
+#
+# Same hard-gold-path mix as cp_0420_cr_trace_mix, but the intermediate
+# board's empty-cell count is drawn per-sample from a Gaussian instead of
+# being a fixed constant. This smooths the per-stage empty-cell distribution
+# so the transition into the natural stage-3 distribution (~54-58 empties)
+# is less abrupt.
+#
+# Build the curriculum datasets once before training:
+#
+# python -m dataset.build_curriculum_dataset \
+#   --source-dir data/sudoku-extreme-1k-aug-1000 \
+#   --output-dir data/sudoku-extreme-1k-aug-1000-stage1-hard-gp-gaussian \
+#   --empty-cells-mean 20 --empty-cells-std 5 --hard-only
+#
+#   python -m dataset.build_curriculum_dataset \
+#     --source-dir data/sudoku-extreme-1k-aug-1000 \
+#     --output-dir data/sudoku-extreme-1k-aug-1000-stage2-hard-gp-gaussian \
+#     --empty-cells-mean 40 --empty-cells-std 5 --hard-only
+#
+# python -m dataset.build_curriculum_dataset \
+#   --source-dir data/sudoku-extreme-1k-aug-1000 \
+#   --output-dir data/sudoku-extreme-1k-aug-1000-stage3-hard-gp-gaussian \
+#   --empty-cells-mean 45 --empty-cells-std 5 --hard-only
+#
+# python -m dataset.build_curriculum_dataset \
+#   --source-dir data/sudoku-extreme-1k-aug-1000 \
+#   --output-dir data/sudoku-extreme-1k-aug-1000-stage4-hard-gp-gaussian \
+#   --empty-cells-mean 50 --empty-cells-std 5 --hard-only
+#
+# Stage 1. hard -&gt; intermediate @ N(20, 5) empty cells; easy/medium unchanged
+# Stage 2. hard -&gt; intermediate @ N(40, 5) empty cells; easy/medium unchanged
+# Stage 3. hard -&gt; intermediate @ N(45, 5) empty cells; easy/medium unchanged
+# Stage 4. hard -&gt; intermediate @ N(50, 5) empty cells; easy/medium unchanged
+# Stage 5. original dataset (no replacement)
+#
+# Usage: bash pretrain_cr.sh exp_0421_cr_trace_mix_gaussian.yaml
+name: exp_0421_cr_trace_mix_gaussian
+depth:
+  H_cycles: 1
+  L_cycles: 2
+  L_layers: 2
+stages:
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage1-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage2-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage3-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000-stage4-hard-gp-gaussian
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+  - data_path: data/sudoku-extreme-1k-aug-1000
+    nsup: 16
+    num_epochs: 10000
+    batch_size: 768
+    eval_interval: 1000
+</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add column 'best exact_acc @ halt_or_nsup 16' (max of eval_strat_nsup16/all_exact_acc_at_halt_or_max)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -458,15 +458,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>best exact_acc @ halt_or_nsup 16</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
@@ -522,15 +527,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F2">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.597177</t>
+        </is>
+      </c>
+      <c r="G2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G2">
+      <c r="H2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H2">
+      <c r="I2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -585,15 +595,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F3">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.687549</t>
+        </is>
+      </c>
+      <c r="G3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G3">
+      <c r="H3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H3">
+      <c r="I3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -670,15 +685,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F4">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.569283</t>
+        </is>
+      </c>
+      <c r="G4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G4">
+      <c r="H4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H4">
+      <c r="I4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -830,15 +850,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F5">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.532132</t>
+        </is>
+      </c>
+      <c r="G5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G5">
+      <c r="H5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -937,15 +962,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F6">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.532612</t>
+        </is>
+      </c>
+      <c r="G6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1009,15 +1039,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F7">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.582091</t>
+        </is>
+      </c>
+      <c r="G7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G7">
+      <c r="H7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1086,15 +1121,20 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F8">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.607629</t>
+        </is>
+      </c>
+      <c r="G8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="G8">
+      <c r="H8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
add column 'best exact_acc @ halt_or_nsup 32' (max of eval_strat_nsup32/all_exact_acc_at_halt_or_max)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -463,15 +463,20 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>best exact_acc @ halt_or_nsup 32</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
@@ -532,15 +537,20 @@
           <t>0.597177</t>
         </is>
       </c>
-      <c r="G2">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.669081</t>
+        </is>
+      </c>
+      <c r="H2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H2">
+      <c r="I2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I2">
+      <c r="J2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -600,15 +610,20 @@
           <t>0.687549</t>
         </is>
       </c>
-      <c r="G3">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.739786</t>
+        </is>
+      </c>
+      <c r="H3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H3">
+      <c r="I3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I3">
+      <c r="J3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -690,15 +705,20 @@
           <t>0.569283</t>
         </is>
       </c>
-      <c r="G4">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.634416</t>
+        </is>
+      </c>
+      <c r="H4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H4">
+      <c r="I4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -855,15 +875,20 @@
           <t>0.532132</t>
         </is>
       </c>
-      <c r="G5">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.594424</t>
+        </is>
+      </c>
+      <c r="H5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -967,15 +992,20 @@
           <t>0.532612</t>
         </is>
       </c>
-      <c r="G6">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.589939</t>
+        </is>
+      </c>
+      <c r="H6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1044,15 +1074,20 @@
           <t>0.582091</t>
         </is>
       </c>
-      <c r="G7">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.644759</t>
+        </is>
+      </c>
+      <c r="H7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1126,15 +1161,20 @@
           <t>0.607629</t>
         </is>
       </c>
-      <c r="G8">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.677068</t>
+        </is>
+      </c>
+      <c r="H8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
add column 'best exact_acc @ halt_or_nsup 64' (max of eval_strat_nsup64/all_exact_acc_at_halt_or_max)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -468,15 +468,20 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>best exact_acc @ halt_or_nsup 64</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
@@ -542,15 +547,20 @@
           <t>0.669081</t>
         </is>
       </c>
-      <c r="H2">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.714752</t>
+        </is>
+      </c>
+      <c r="I2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I2">
+      <c r="J2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J2">
+      <c r="K2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -615,15 +625,20 @@
           <t>0.739786</t>
         </is>
       </c>
-      <c r="H3">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.775009</t>
+        </is>
+      </c>
+      <c r="I3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I3">
+      <c r="J3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J3">
+      <c r="K3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -710,15 +725,20 @@
           <t>0.634416</t>
         </is>
       </c>
-      <c r="H4">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.675512</t>
+        </is>
+      </c>
+      <c r="I4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J4">
+      <c r="K4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -880,15 +900,20 @@
           <t>0.594424</t>
         </is>
       </c>
-      <c r="H5">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.629888</t>
+        </is>
+      </c>
+      <c r="I5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J5">
+      <c r="K5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -997,15 +1022,20 @@
           <t>0.589939</t>
         </is>
       </c>
-      <c r="H6">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.622826</t>
+        </is>
+      </c>
+      <c r="I6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="K6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1079,15 +1109,20 @@
           <t>0.644759</t>
         </is>
       </c>
-      <c r="H7">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.680964</t>
+        </is>
+      </c>
+      <c r="I7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="K7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
@@ -1166,15 +1201,20 @@
           <t>0.677068</t>
         </is>
       </c>
-      <c r="H8">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.722150</t>
+        </is>
+      </c>
+      <c r="I8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="K8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
backfill missing photo columns from PHOTO_COLUMNS
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -486,6 +486,11 @@
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>train_exact_accuracy</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -564,6 +569,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L2">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -642,6 +651,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L3">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="100" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -742,6 +755,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L4">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -917,6 +934,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L5">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -1039,6 +1060,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L6">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="100" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -1126,6 +1151,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L7">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="100" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -1218,6 +1247,10 @@
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
+      <c r="L8">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add column 'best train/exact_accuracy' (max of train/exact_accuracy)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -473,20 +473,25 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>best train/exact_accuracy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>exact_acc @ halt_or_nsup 16</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 32</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>exact_acc @ halt_or_nsup 64</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>train_exact_accuracy</t>
         </is>
@@ -557,19 +562,24 @@
           <t>0.714752</t>
         </is>
       </c>
-      <c r="I2">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.865672</t>
+        </is>
+      </c>
+      <c r="J2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J2">
+      <c r="K2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K2">
+      <c r="L2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L2">
+      <c r="M2">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0413_baseline_220918_stage2/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -639,19 +649,24 @@
           <t>0.775009</t>
         </is>
       </c>
-      <c r="I3">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.714286</t>
+        </is>
+      </c>
+      <c r="J3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J3">
+      <c r="K3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K3">
+      <c r="L3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L3">
+      <c r="M3">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0419_cr_baseline_004937_stage2/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -743,19 +758,24 @@
           <t>0.675512</t>
         </is>
       </c>
-      <c r="I4">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.766355</t>
+        </is>
+      </c>
+      <c r="J4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J4">
+      <c r="K4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K4">
+      <c r="L4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L4">
+      <c r="M4">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0413_cr_trace_mix_gaussian_210715_stage2/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -922,19 +942,24 @@
           <t>0.629888</t>
         </is>
       </c>
-      <c r="I5">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1.000000</t>
+        </is>
+      </c>
+      <c r="J5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J5">
+      <c r="K5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K5">
+      <c r="L5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L5">
+      <c r="M5">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0420_cr_trace_mix_gaussian_dense_141633_stage20/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -1048,19 +1073,24 @@
           <t>0.622826</t>
         </is>
       </c>
-      <c r="I6">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.814433</t>
+        </is>
+      </c>
+      <c r="J6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="K6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K6">
+      <c r="L6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0421_cr_trace_mix_gaussian_192914_stage4/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -1139,19 +1169,24 @@
           <t>0.680964</t>
         </is>
       </c>
-      <c r="I7">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.685185</t>
+        </is>
+      </c>
+      <c r="J7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="K7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K7">
+      <c r="L7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L7">
+      <c r="M7">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_004417_stage2/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
@@ -1235,19 +1270,24 @@
           <t>0.722150</t>
         </is>
       </c>
-      <c r="I8">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.865979</t>
+        </is>
+      </c>
+      <c r="J8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="K8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="K8">
+      <c r="L8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="L8">
+      <c r="M8">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/exp_0414_bt_descendents_015622_stage2/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
add column 'train/exact_accuracy (last 1000 avg)' (tail_mean(1000) of train/exact_accuracy); dropped ['best train/exact_accuracy']
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>best train/exact_accuracy</t>
+          <t>train/exact_accuracy (last 1000 avg)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.814373</t>
         </is>
       </c>
       <c r="J2">
@@ -651,7 +651,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.573716</t>
         </is>
       </c>
       <c r="J3">
@@ -760,7 +760,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.536861</t>
         </is>
       </c>
       <c r="J4">
@@ -944,7 +944,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.511622</t>
         </is>
       </c>
       <c r="J5">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.468834</t>
         </is>
       </c>
       <c r="J6">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.575606</t>
         </is>
       </c>
       <c r="J7">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.000000</t>
+          <t>0.734369</t>
         </is>
       </c>
       <c r="J8">

</xml_diff>

<commit_message>
add 1 run(s) to index: cr_0429_derive_ignore_hybrid_224622
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1292,6 +1292,38 @@
         <v/>
       </c>
     </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_hybrid_224622</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>16</v>
+      </c>
+      <c r="E9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add 1 run(s) to index: cr_0429_derive_ignore_194437
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1324,6 +1324,38 @@
         <v/>
       </c>
     </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_194437</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add 1 run(s) to index: cr_0429_derive_ignore_v2_154835
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -547,9 +547,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>0.814373</t>
@@ -622,9 +619,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>0.573716</t>
@@ -719,9 +713,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>0.536861</t>
@@ -891,9 +882,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>0.511622</t>
@@ -1010,9 +998,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>0.468834</t>
@@ -1094,9 +1079,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>0.575606</t>
@@ -1183,9 +1165,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>0.734369</t>
@@ -1249,11 +1228,6 @@
           <t>0.030640</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -1296,11 +1270,38 @@
           <t>0.608554</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_v2_154835</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add 1 run(s) to index: cr_0429_derive_ignore_m3_194001
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1303,6 +1303,38 @@
         <v/>
       </c>
     </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_m3_194001</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix column alignment for v2/m3 rows — photos now in correct columns 10-13, best metrics in 6-8
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1277,30 +1277,57 @@
           <t>cr_0429_derive_ignore_v2_154835</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.715665</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.678776</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.616707</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1">
@@ -1309,30 +1336,57 @@
           <t>cr_0429_derive_ignore_m3_194001</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>16</v>
-      </c>
-      <c r="E12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="F12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="G12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.664019</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.631632</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.575769</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix v2/m3 row alignment — H_cycles/L_cycles/max_halt_steps now in correct columns 3/4/5 (config col empty)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1277,22 +1277,22 @@
           <t>cr_0429_derive_ignore_v2_154835</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>0.715665</t>
@@ -1309,25 +1309,21 @@
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png</t>
-        </is>
+      <c r="J11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1">
@@ -1336,22 +1332,22 @@
           <t>cr_0429_derive_ignore_m3_194001</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>0.664019</t>
@@ -1368,25 +1364,21 @@
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png</t>
-        </is>
+      <c r="J12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fully realign all cr_0429 rows to header — H/L/max in cols 3/4/5, all 4 photo slots filled, train_acc avg from wandb
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1200,19 +1200,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>0.093499</t>
@@ -1227,6 +1227,27 @@
         <is>
           <t>0.030640</t>
         </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.580174</t>
+        </is>
+      </c>
+      <c r="J9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="100" customHeight="1">
@@ -1242,19 +1263,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>0.704030</t>
@@ -1269,6 +1290,27 @@
         <is>
           <t>0.608554</t>
         </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.868711</t>
+        </is>
+      </c>
+      <c r="J10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="100" customHeight="1">
@@ -1277,7 +1319,6 @@
           <t>cr_0429_derive_ignore_v2_154835</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>1</t>
@@ -1308,7 +1349,11 @@
           <t>0.616707</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.885604</t>
+        </is>
+      </c>
       <c r="J11">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
@@ -1332,7 +1377,6 @@
           <t>cr_0429_derive_ignore_m3_194001</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>1</t>
@@ -1363,7 +1407,11 @@
           <t>0.575769</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.506661</t>
+        </is>
+      </c>
       <c r="J12">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>

</xml_diff>

<commit_message>
remove cr_0429_derive_ignore_hybrid_224622 from index — failed run, not publishable
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1190,7 +1190,7 @@
     <row r="9" ht="100" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cr_0429_derive_ignore_hybrid_224622</t>
+          <t>cr_0429_derive_ignore_194437</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1215,57 +1215,52 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.093499</t>
+          <t>0.704030</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.075215</t>
+          <t>0.668026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.030640</t>
+          <t>0.608554</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.580174</t>
+          <t>0.868711</t>
         </is>
       </c>
       <c r="J9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
       <c r="K9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
       <c r="L9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
       <c r="M9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_hybrid_224622_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cr_0429_derive_ignore_194437</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+          <t>cr_0429_derive_ignore_v2_154835</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>2</t>
@@ -1278,45 +1273,45 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.704030</t>
+          <t>0.715665</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.668026</t>
+          <t>0.678776</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.608554</t>
+          <t>0.616707</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.868711</t>
+          <t>0.885604</t>
         </is>
       </c>
       <c r="J10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
       <c r="K10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
       <c r="L10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
       <c r="M10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="100" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cr_0429_derive_ignore_v2_154835</t>
+          <t>cr_0429_derive_ignore_m3_194001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1336,99 +1331,42 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.715665</t>
+          <t>0.664019</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.678776</t>
+          <t>0.631632</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0.616707</t>
+          <t>0.575769</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.885604</t>
+          <t>0.506661</t>
         </is>
       </c>
       <c r="J11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
       <c r="K11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
       <c r="L11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
       <c r="M11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="100" customHeight="1">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>cr_0429_derive_ignore_m3_194001</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0.664019</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0.631632</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0.575769</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.506661</t>
-        </is>
-      </c>
-      <c r="J12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="K12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="L12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="M12">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="12" ht="100" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
backfill best exact_acc @ halt_or_nsup 16/32/64 for 7 older runs from local snapshot/CSV data
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -547,6 +547,21 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.714752</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.669081</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.597177</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>0.814373</t>
@@ -619,6 +634,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.529864</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>0.573716</t>
@@ -713,6 +733,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.569215</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>0.536861</t>
@@ -882,6 +907,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.531810</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>0.511622</t>
@@ -998,6 +1028,21 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.622826</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.589939</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.532612</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>0.468834</t>
@@ -1079,6 +1124,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.582195</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>0.575606</t>
@@ -1165,6 +1215,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.607816</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>0.734369</t>

</xml_diff>

<commit_message>
backfill best @ n=16/32/64 for all rows from wandb eval_strat_nsup* namespace
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -634,9 +634,19 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.775009</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.739786</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.529864</t>
+          <t>0.687549</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -733,9 +743,19 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.675512</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.634416</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.569215</t>
+          <t>0.569283</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -907,6 +927,16 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.628980</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.594275</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>0.531810</t>
@@ -1124,6 +1154,16 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.680964</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.644759</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>0.582195</t>
@@ -1215,6 +1255,16 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.722150</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.677068</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>0.607816</t>
@@ -1270,17 +1320,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.704030</t>
+          <t>0.719288</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.668026</t>
+          <t>0.681120</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.608554</t>
+          <t>0.618053</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">

</xml_diff>

<commit_message>
consolidate cr_0429_derive_ignore seeds → one row with mean±std + band plots
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1295,19 +1295,15 @@
     <row r="9" ht="100" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cr_0429_derive_ignore_194437</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+          <t>cr_0429_derive_ignore (2-seed avg)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>2</t>
@@ -1320,157 +1316,43 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.719288</t>
+          <t>0.7164 ± 0.0041</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.681120</t>
+          <t>0.6790 ± 0.0030</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.618053</t>
+          <t>0.6168 ± 0.0018</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.868711</t>
+          <t>0.9042 ± 0.0122</t>
         </is>
       </c>
       <c r="J9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
       <c r="K9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
       <c r="L9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
       <c r="M9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_194437_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>cr_0429_derive_ignore_v2_154835</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>0.715665</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0.678776</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0.616707</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.885604</t>
-        </is>
-      </c>
-      <c r="J10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="K10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="L10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="M10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_v2_154835_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="100" customHeight="1">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>cr_0429_derive_ignore_m3_194001</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>0.664019</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0.631632</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0.575769</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.506661</t>
-        </is>
-      </c>
-      <c r="J11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="K11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="L11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="M11">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="10" ht="100" customHeight="1"/>
+    <row r="11" ht="100" customHeight="1"/>
     <row r="12" ht="100" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add 1 run(s) to index: cr_0429_derive_ignore_m2_204257
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1298,7 +1298,6 @@
           <t>cr_0429_derive_ignore (2-seed avg)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -1351,7 +1350,43 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1"/>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_m2_204257</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M10">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
     <row r="11" ht="100" customHeight="1"/>
     <row r="12" ht="100" customHeight="1"/>
   </sheetData>

</xml_diff>

<commit_message>
fill M2 best metrics + train_avg from wandb
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -1356,7 +1356,6 @@
           <t>cr_0429_derive_ignore_m2_204257</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>1</v>
       </c>
@@ -1366,10 +1365,26 @@
       <c r="E10" t="n">
         <v>16</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.254767</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.244821</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.225343</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.167461</t>
+        </is>
+      </c>
       <c r="J10">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>

</xml_diff>

<commit_message>
remove M2 from index; add missing M3 row to XLSX (was only in CSV)
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1295,9 +1295,10 @@
     <row r="9" ht="100" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cr_0429_derive_ignore (2-seed avg)</t>
-        </is>
-      </c>
+          <t>cr_0429_derive_ignore_m3_194001</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -1315,93 +1316,42 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.7164 ± 0.0041</t>
+          <t>0.664019</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.6790 ± 0.0030</t>
+          <t>0.631632</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.6168 ± 0.0018</t>
+          <t>0.575769</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.9042 ± 0.0122</t>
+          <t>0.506661</t>
         </is>
       </c>
       <c r="J9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
       <c r="K9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
       <c r="L9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
       <c r="M9">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/train_exact_accuracy.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>cr_0429_derive_ignore_m2_204257</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>16</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>0.254767</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0.244821</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0.225343</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.167461</t>
-        </is>
-      </c>
-      <c r="J10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
-        <v/>
-      </c>
-      <c r="K10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
-        <v/>
-      </c>
-      <c r="L10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
-        <v/>
-      </c>
-      <c r="M10">
-        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m2_204257_stage0/training_dynamics/train_exact_accuracy.png")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="10" ht="100" customHeight="1"/>
     <row r="11" ht="100" customHeight="1"/>
     <row r="12" ht="100" customHeight="1"/>
   </sheetData>

</xml_diff>

<commit_message>
regenerate XLSX from CSV — restore (2-seed avg) row that was accidentally overwritten
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -503,7 +503,7 @@
           <t>cr_0413_baseline_220918</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t xml:space="preserve"># Baseline, no CR on depth, no CR on data
 #
@@ -590,7 +590,7 @@
           <t>exp_0419_cr_baseline_004937</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t xml:space="preserve"># Baseline, no CR on depth, no CR on data
 #
@@ -677,7 +677,7 @@
           <t>exp_0413_cr_trace_mix_gaussian_210715</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t xml:space="preserve"># Curriculum learning config (gaussian variant).
 #
@@ -786,7 +786,7 @@
           <t>exp_0420_cr_trace_mix_gaussian_dense_141633</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t xml:space="preserve"># Curriculum learning config (gaussian, dense variant).
 #
@@ -970,7 +970,7 @@
           <t>exp_0421_cr_trace_mix_gaussian_192914</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve"># Curriculum learning config (gaussian variant).
 #
@@ -1101,7 +1101,7 @@
           <t>exp_0414_bt_004417</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t xml:space="preserve"># Curriculum learning config (BT)
 #
@@ -1197,7 +1197,7 @@
           <t>exp_0414_bt_descendents_015622</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t xml:space="preserve"># Curriculum learning config (BT by wrong-subtree depth, hard-only replacement)
 #
@@ -1295,63 +1295,119 @@
     <row r="9" ht="100" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
+          <t>cr_0429_derive_ignore (2-seed avg)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.7164 ± 0.0041</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.6790 ± 0.0030</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.6168 ± 0.0018</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.9042 ± 0.0122</t>
+        </is>
+      </c>
+      <c r="J9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_2seeds_combined/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>cr_0429_derive_ignore_m3_194001</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>0.664019</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>0.631632</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>0.575769</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>0.506661</t>
         </is>
       </c>
-      <c r="J9">
+      <c r="J10">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
         <v/>
       </c>
-      <c r="K9">
+      <c r="K10">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
         <v/>
       </c>
-      <c r="L9">
+      <c r="L10">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
         <v/>
       </c>
-      <c r="M9">
+      <c r="M10">
         <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_m3_194001_stage0/training_dynamics/train_exact_accuracy.png")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1"/>
     <row r="11" ht="100" customHeight="1"/>
     <row r="12" ht="100" customHeight="1"/>
   </sheetData>

</xml_diff>

<commit_message>
add 3 run(s) to index: cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241, cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102, cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -1408,8 +1408,99 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="100" customHeight="1"/>
-    <row r="12" ht="100" customHeight="1"/>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M11">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_divsup_lam015_aux00_smoke_093241_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M12">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust90_wcsoft2_divsup_lam015_aux00_smoke_094102_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244_stage0/training_dynamics/exact_acc_at_halt_or_nsup16.png")</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244_stage0/training_dynamics/exact_acc_at_halt_or_nsup32.png")</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244_stage0/training_dynamics/exact_acc_at_halt_or_nsup64.png")</f>
+        <v/>
+      </c>
+      <c r="M13">
+        <f>IMAGE("https://raw.githubusercontent.com/yoyostudy/trm-cr-experiment-photos/cr_0429_derive_ignore_trust95_wcsoft2_div81_lam015_aux00_smoke_093244_stage0/training_dynamics/train_exact_accuracy.png")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>